<commit_message>
Retag HUD HomeStore as HUD Home (blue pin); refresh xlsx
HUD HomeStore is HUD government-owned inventory, not private bank REO.
The map legend treats "HUD / HomePath" (blue) and "REO / Bank-Owned"
(red) as separate categories for exactly this reason. We were
misclassifying the 29 HUD HomeStore properties as generic REO.

Fix in hud_reo.py: set listingType = "HUD Home" so they render blue.
Backfilled data/foreclosures_va.json so the color change takes effect
on the live site immediately (no workflow wait).

Also refreshed data/hud_va.xlsx with the user's latest HUD HomeStore
case list export (4_21_2026_Case_List.xlsx, 28 VA rows).

Note: the fresh export is VA-only; to show MD HUD REO on the map,
a separate MD case list would need to be exported from HUD HomeStore
and merged. The scraper already accepts VA + MD state rows.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/hud_va.xlsx
+++ b/data/hud_va.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="481" uniqueCount="264">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="465" uniqueCount="258">
   <si>
     <t>Property Case</t>
   </si>
@@ -101,210 +101,213 @@
     <t>04/06/2026</t>
   </si>
   <si>
+    <t>04/22/2026</t>
+  </si>
+  <si>
+    <t>Extended</t>
+  </si>
+  <si>
+    <t>Price Reduced</t>
+  </si>
+  <si>
+    <t>07/12/2026</t>
+  </si>
+  <si>
+    <t>548-479514</t>
+  </si>
+  <si>
+    <t>9865 High Water Ct</t>
+  </si>
+  <si>
+    <t>Burke</t>
+  </si>
+  <si>
+    <t>22015</t>
+  </si>
+  <si>
+    <t>Fairfax</t>
+  </si>
+  <si>
+    <t>2.5</t>
+  </si>
+  <si>
+    <t>1407</t>
+  </si>
+  <si>
+    <t>1979</t>
+  </si>
+  <si>
+    <t>IE (Insured Escrow)</t>
+  </si>
+  <si>
+    <t>04/14/2026</t>
+  </si>
+  <si>
+    <t>04/24/2026</t>
+  </si>
+  <si>
+    <t>Exclusive</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>04/28/2026</t>
+  </si>
+  <si>
+    <t>541-918384</t>
+  </si>
+  <si>
+    <t>4216 Rosewood Ct</t>
+  </si>
+  <si>
+    <t>Williamsburg</t>
+  </si>
+  <si>
+    <t>23188</t>
+  </si>
+  <si>
+    <t>James City</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>1871</t>
+  </si>
+  <si>
+    <t>1996</t>
+  </si>
+  <si>
+    <t>04/09/2026</t>
+  </si>
+  <si>
+    <t>04/23/2026</t>
+  </si>
+  <si>
+    <t>544-354760</t>
+  </si>
+  <si>
+    <t>513 Water Lilly Rd</t>
+  </si>
+  <si>
+    <t>Portsmouth</t>
+  </si>
+  <si>
+    <t>23701</t>
+  </si>
+  <si>
+    <t>Portsmouth City</t>
+  </si>
+  <si>
+    <t>2305</t>
+  </si>
+  <si>
+    <t>2006</t>
+  </si>
+  <si>
+    <t>03/03/2026</t>
+  </si>
+  <si>
+    <t>09/18/2026</t>
+  </si>
+  <si>
+    <t>544-312353</t>
+  </si>
+  <si>
+    <t>2216 Deep Creek Blv</t>
+  </si>
+  <si>
+    <t>23704</t>
+  </si>
+  <si>
+    <t>2483</t>
+  </si>
+  <si>
+    <t>1961</t>
+  </si>
+  <si>
+    <t>08/04/2026</t>
+  </si>
+  <si>
+    <t>544-379898</t>
+  </si>
+  <si>
+    <t>3415 Willis Wharf Rd</t>
+  </si>
+  <si>
+    <t>Exmore</t>
+  </si>
+  <si>
+    <t>23350</t>
+  </si>
+  <si>
+    <t>Northampton</t>
+  </si>
+  <si>
+    <t>2753</t>
+  </si>
+  <si>
+    <t>1968</t>
+  </si>
+  <si>
+    <t>06/20/2026</t>
+  </si>
+  <si>
+    <t>544-326749</t>
+  </si>
+  <si>
+    <t>113 W Main Street</t>
+  </si>
+  <si>
+    <t>Wakefield</t>
+  </si>
+  <si>
+    <t>23888</t>
+  </si>
+  <si>
+    <t>Sussex</t>
+  </si>
+  <si>
+    <t>3.5</t>
+  </si>
+  <si>
+    <t>2724</t>
+  </si>
+  <si>
+    <t>1900</t>
+  </si>
+  <si>
+    <t>03/30/2026</t>
+  </si>
+  <si>
+    <t>09/25/2026</t>
+  </si>
+  <si>
+    <t>544-371294</t>
+  </si>
+  <si>
+    <t>20132 King William Rd</t>
+  </si>
+  <si>
+    <t>King William</t>
+  </si>
+  <si>
+    <t>23086</t>
+  </si>
+  <si>
+    <t>1827</t>
+  </si>
+  <si>
+    <t>2022</t>
+  </si>
+  <si>
+    <t>04/07/2026</t>
+  </si>
+  <si>
     <t>04/21/2026</t>
   </si>
   <si>
-    <t>Extended</t>
-  </si>
-  <si>
-    <t>Price Reduced</t>
-  </si>
-  <si>
-    <t>07/12/2026</t>
-  </si>
-  <si>
-    <t>548-479514</t>
-  </si>
-  <si>
-    <t>9865 High Water Ct</t>
-  </si>
-  <si>
-    <t>Burke</t>
-  </si>
-  <si>
-    <t>22015</t>
-  </si>
-  <si>
-    <t>Fairfax</t>
-  </si>
-  <si>
-    <t>2.5</t>
-  </si>
-  <si>
-    <t>1407</t>
-  </si>
-  <si>
-    <t>1979</t>
-  </si>
-  <si>
-    <t>IE (Insured Escrow)</t>
-  </si>
-  <si>
-    <t>04/14/2026</t>
-  </si>
-  <si>
-    <t>04/24/2026</t>
-  </si>
-  <si>
-    <t>Exclusive</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>04/28/2026</t>
-  </si>
-  <si>
-    <t>541-918384</t>
-  </si>
-  <si>
-    <t>4216 Rosewood Ct</t>
-  </si>
-  <si>
-    <t>Williamsburg</t>
-  </si>
-  <si>
-    <t>23188</t>
-  </si>
-  <si>
-    <t>James City</t>
-  </si>
-  <si>
-    <t>4</t>
-  </si>
-  <si>
-    <t>1871</t>
-  </si>
-  <si>
-    <t>1996</t>
-  </si>
-  <si>
-    <t>04/09/2026</t>
-  </si>
-  <si>
-    <t>04/23/2026</t>
-  </si>
-  <si>
-    <t>544-354760</t>
-  </si>
-  <si>
-    <t>513 Water Lilly Rd</t>
-  </si>
-  <si>
-    <t>Portsmouth</t>
-  </si>
-  <si>
-    <t>23701</t>
-  </si>
-  <si>
-    <t>Portsmouth City</t>
-  </si>
-  <si>
-    <t>2305</t>
-  </si>
-  <si>
-    <t>2006</t>
-  </si>
-  <si>
-    <t>03/03/2026</t>
-  </si>
-  <si>
-    <t>09/18/2026</t>
-  </si>
-  <si>
-    <t>544-312353</t>
-  </si>
-  <si>
-    <t>2216 Deep Creek Blv</t>
-  </si>
-  <si>
-    <t>23704</t>
-  </si>
-  <si>
-    <t>2483</t>
-  </si>
-  <si>
-    <t>1961</t>
-  </si>
-  <si>
-    <t>08/04/2026</t>
-  </si>
-  <si>
-    <t>544-379898</t>
-  </si>
-  <si>
-    <t>3415 Willis Wharf Rd</t>
-  </si>
-  <si>
-    <t>Exmore</t>
-  </si>
-  <si>
-    <t>23350</t>
-  </si>
-  <si>
-    <t>Northampton</t>
-  </si>
-  <si>
-    <t>2753</t>
-  </si>
-  <si>
-    <t>1968</t>
-  </si>
-  <si>
-    <t>06/20/2026</t>
-  </si>
-  <si>
-    <t>544-326749</t>
-  </si>
-  <si>
-    <t>113 W Main Street</t>
-  </si>
-  <si>
-    <t>Wakefield</t>
-  </si>
-  <si>
-    <t>23888</t>
-  </si>
-  <si>
-    <t>Sussex</t>
-  </si>
-  <si>
-    <t>3.5</t>
-  </si>
-  <si>
-    <t>2724</t>
-  </si>
-  <si>
-    <t>1900</t>
-  </si>
-  <si>
-    <t>03/30/2026</t>
-  </si>
-  <si>
-    <t>09/25/2026</t>
-  </si>
-  <si>
-    <t>544-371294</t>
-  </si>
-  <si>
-    <t>20132 King William Rd</t>
-  </si>
-  <si>
-    <t>King William</t>
-  </si>
-  <si>
-    <t>23086</t>
-  </si>
-  <si>
-    <t>1827</t>
-  </si>
-  <si>
-    <t>2022</t>
-  </si>
-  <si>
-    <t>04/07/2026</t>
-  </si>
-  <si>
     <t>544-379883</t>
   </si>
   <si>
@@ -321,27 +324,6 @@
   </si>
   <si>
     <t>1976</t>
-  </si>
-  <si>
-    <t>544-360655</t>
-  </si>
-  <si>
-    <t>54 Burtis Street</t>
-  </si>
-  <si>
-    <t>23702</t>
-  </si>
-  <si>
-    <t>1658</t>
-  </si>
-  <si>
-    <t>1929</t>
-  </si>
-  <si>
-    <t>02/27/2026</t>
-  </si>
-  <si>
-    <t>08/25/2026</t>
   </si>
   <si>
     <t>544-235586</t>
@@ -1276,27 +1258,27 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{fa744ca9-2541-490d-859f-53aa9b18c23a}">
-  <dimension ref="A1:Q30"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{cb343c31-987c-4120-bda3-2ef8949a693b}">
+  <dimension ref="A1:Q29"/>
   <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="1" width="16.857142857142858" customWidth="1"/>
-    <col min="2" max="2" width="23.142857142857142" customWidth="1"/>
-    <col min="3" max="3" width="14.857142857142858" customWidth="1"/>
-    <col min="4" max="4" width="7.571428571428571" customWidth="1"/>
-    <col min="5" max="5" width="11" customWidth="1"/>
-    <col min="6" max="6" width="17.857142857142858" customWidth="1"/>
+    <col min="2" max="2" width="21.857142857142858" customWidth="1"/>
+    <col min="3" max="3" width="13.857142857142858" customWidth="1"/>
+    <col min="4" max="4" width="7.428571428571429" customWidth="1"/>
+    <col min="5" max="5" width="11.428571428571429" customWidth="1"/>
+    <col min="6" max="6" width="16.142857142857142" customWidth="1"/>
     <col min="7" max="7" width="7.714285714285714" customWidth="1"/>
-    <col min="8" max="8" width="5.857142857142857" customWidth="1"/>
-    <col min="9" max="9" width="7" customWidth="1"/>
-    <col min="10" max="10" width="18.285714285714285" customWidth="1"/>
-    <col min="11" max="11" width="12.714285714285714" customWidth="1"/>
-    <col min="12" max="12" width="17.571428571428573" customWidth="1"/>
-    <col min="13" max="13" width="11.571428571428571" customWidth="1"/>
-    <col min="14" max="14" width="17.142857142857142" customWidth="1"/>
-    <col min="15" max="15" width="16.714285714285715" customWidth="1"/>
-    <col min="16" max="16" width="13" customWidth="1"/>
-    <col min="17" max="17" width="18.571428571428573" customWidth="1"/>
+    <col min="8" max="8" width="6" customWidth="1"/>
+    <col min="9" max="9" width="6.714285714285714" customWidth="1"/>
+    <col min="10" max="10" width="18.714285714285715" customWidth="1"/>
+    <col min="11" max="11" width="12.142857142857142" customWidth="1"/>
+    <col min="12" max="12" width="17" customWidth="1"/>
+    <col min="13" max="13" width="11.285714285714286" customWidth="1"/>
+    <col min="14" max="14" width="17.285714285714285" customWidth="1"/>
+    <col min="15" max="15" width="16.428571428571427" customWidth="1"/>
+    <col min="16" max="16" width="12.285714285714286" customWidth="1"/>
+    <col min="17" max="17" width="18.714285714285715" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="12.75">
@@ -1773,27 +1755,27 @@
         <v>44</v>
       </c>
       <c r="Q9" s="3" t="s">
-        <v>28</v>
+        <v>96</v>
       </c>
     </row>
     <row r="10" spans="1:17" ht="12.75">
       <c r="A10" s="3" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D10" s="3" t="s">
         <v>20</v>
       </c>
       <c r="E10" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="F10" s="3" t="s">
         <v>99</v>
-      </c>
-      <c r="F10" s="3" t="s">
-        <v>98</v>
       </c>
       <c r="G10" s="4">
         <v>296000</v>
@@ -1805,10 +1787,10 @@
         <v>37</v>
       </c>
       <c r="J10" s="3" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="K10" s="3" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="L10" s="3" t="s">
         <v>40</v>
@@ -1831,43 +1813,43 @@
     </row>
     <row r="11" spans="1:17" ht="12.75">
       <c r="A11" s="3" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>58</v>
+        <v>105</v>
       </c>
       <c r="D11" s="3" t="s">
         <v>20</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>60</v>
+        <v>107</v>
       </c>
       <c r="G11" s="4">
-        <v>286000</v>
+        <v>277000</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>51</v>
+        <v>22</v>
       </c>
       <c r="I11" s="3" t="s">
-        <v>37</v>
+        <v>22</v>
       </c>
       <c r="J11" s="3" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="K11" s="3" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="L11" s="3" t="s">
         <v>26</v>
       </c>
       <c r="M11" s="3" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="N11" s="3" t="s">
         <v>28</v>
@@ -1879,27 +1861,27 @@
         <v>44</v>
       </c>
       <c r="Q11" s="3" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
     </row>
     <row r="12" spans="1:17" ht="12.75">
       <c r="A12" s="3" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="D12" s="3" t="s">
         <v>20</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="G12" s="4">
         <v>277000</v>
@@ -1908,178 +1890,178 @@
         <v>22</v>
       </c>
       <c r="I12" s="3" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="J12" s="3" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="K12" s="3" t="s">
-        <v>115</v>
+        <v>53</v>
       </c>
       <c r="L12" s="3" t="s">
         <v>26</v>
       </c>
       <c r="M12" s="3" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="N12" s="3" t="s">
-        <v>28</v>
+        <v>118</v>
       </c>
       <c r="O12" s="3" t="s">
-        <v>29</v>
+        <v>43</v>
       </c>
       <c r="P12" s="3" t="s">
-        <v>44</v>
+        <v>119</v>
       </c>
       <c r="Q12" s="3" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
     </row>
     <row r="13" spans="1:17" ht="12.75">
       <c r="A13" s="3" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="D13" s="3" t="s">
         <v>20</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="G13" s="4">
-        <v>277000</v>
+        <v>264000</v>
       </c>
       <c r="H13" s="3" t="s">
         <v>22</v>
       </c>
       <c r="I13" s="3" t="s">
-        <v>23</v>
+        <v>126</v>
       </c>
       <c r="J13" s="3" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="K13" s="3" t="s">
-        <v>53</v>
+        <v>128</v>
       </c>
       <c r="L13" s="3" t="s">
-        <v>26</v>
+        <v>40</v>
       </c>
       <c r="M13" s="3" t="s">
-        <v>123</v>
+        <v>54</v>
       </c>
       <c r="N13" s="3" t="s">
-        <v>124</v>
+        <v>28</v>
       </c>
       <c r="O13" s="3" t="s">
         <v>43</v>
       </c>
       <c r="P13" s="3" t="s">
-        <v>125</v>
+        <v>44</v>
       </c>
       <c r="Q13" s="3" t="s">
-        <v>126</v>
+        <v>55</v>
       </c>
     </row>
     <row r="14" spans="1:17" ht="12.75">
       <c r="A14" s="3" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="D14" s="3" t="s">
         <v>20</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="G14" s="4">
-        <v>264000</v>
+        <v>255000</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="I14" s="3" t="s">
-        <v>132</v>
+        <v>23</v>
       </c>
       <c r="J14" s="3" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="K14" s="3" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="L14" s="3" t="s">
-        <v>40</v>
+        <v>26</v>
       </c>
       <c r="M14" s="3" t="s">
-        <v>54</v>
+        <v>136</v>
       </c>
       <c r="N14" s="3" t="s">
         <v>28</v>
       </c>
       <c r="O14" s="3" t="s">
-        <v>43</v>
+        <v>29</v>
       </c>
       <c r="P14" s="3" t="s">
         <v>44</v>
       </c>
       <c r="Q14" s="3" t="s">
-        <v>55</v>
+        <v>137</v>
       </c>
     </row>
     <row r="15" spans="1:17" ht="12.75">
       <c r="A15" s="3" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="D15" s="3" t="s">
         <v>20</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="G15" s="4">
-        <v>255000</v>
+        <v>252000</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="I15" s="3" t="s">
-        <v>23</v>
+        <v>143</v>
       </c>
       <c r="J15" s="3" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="K15" s="3" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="L15" s="3" t="s">
         <v>26</v>
       </c>
       <c r="M15" s="3" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="N15" s="3" t="s">
         <v>28</v>
@@ -2088,51 +2070,51 @@
         <v>29</v>
       </c>
       <c r="P15" s="3" t="s">
-        <v>44</v>
+        <v>30</v>
       </c>
       <c r="Q15" s="3" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
     </row>
     <row r="16" spans="1:17" ht="12.75">
       <c r="A16" s="3" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="D16" s="3" t="s">
         <v>20</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="G16" s="4">
-        <v>252000</v>
+        <v>221000</v>
       </c>
       <c r="H16" s="3" t="s">
         <v>22</v>
       </c>
       <c r="I16" s="3" t="s">
-        <v>149</v>
+        <v>126</v>
       </c>
       <c r="J16" s="3" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="K16" s="3" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="L16" s="3" t="s">
         <v>26</v>
       </c>
       <c r="M16" s="3" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="N16" s="3" t="s">
         <v>28</v>
@@ -2141,51 +2123,51 @@
         <v>29</v>
       </c>
       <c r="P16" s="3" t="s">
-        <v>30</v>
+        <v>44</v>
       </c>
       <c r="Q16" s="3" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
     </row>
     <row r="17" spans="1:17" ht="12.75">
       <c r="A17" s="3" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="D17" s="3" t="s">
         <v>20</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="G17" s="4">
-        <v>221000</v>
+        <v>209000</v>
       </c>
       <c r="H17" s="3" t="s">
         <v>22</v>
       </c>
       <c r="I17" s="3" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="J17" s="3" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="K17" s="3" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="L17" s="3" t="s">
-        <v>26</v>
+        <v>40</v>
       </c>
       <c r="M17" s="3" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="N17" s="3" t="s">
         <v>28</v>
@@ -2197,48 +2179,48 @@
         <v>44</v>
       </c>
       <c r="Q17" s="3" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
     </row>
     <row r="18" spans="1:17" ht="12.75">
       <c r="A18" s="3" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>165</v>
+        <v>150</v>
       </c>
       <c r="D18" s="3" t="s">
         <v>20</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>167</v>
+        <v>152</v>
       </c>
       <c r="G18" s="4">
-        <v>209000</v>
+        <v>205000</v>
       </c>
       <c r="H18" s="3" t="s">
-        <v>22</v>
+        <v>51</v>
       </c>
       <c r="I18" s="3" t="s">
-        <v>132</v>
+        <v>23</v>
       </c>
       <c r="J18" s="3" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="K18" s="3" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="L18" s="3" t="s">
         <v>40</v>
       </c>
       <c r="M18" s="3" t="s">
-        <v>170</v>
+        <v>27</v>
       </c>
       <c r="N18" s="3" t="s">
         <v>28</v>
@@ -2247,7 +2229,7 @@
         <v>29</v>
       </c>
       <c r="P18" s="3" t="s">
-        <v>44</v>
+        <v>30</v>
       </c>
       <c r="Q18" s="3" t="s">
         <v>171</v>
@@ -2261,37 +2243,37 @@
         <v>173</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>156</v>
+        <v>174</v>
       </c>
       <c r="D19" s="3" t="s">
         <v>20</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>158</v>
+        <v>83</v>
       </c>
       <c r="G19" s="4">
-        <v>205000</v>
+        <v>193000</v>
       </c>
       <c r="H19" s="3" t="s">
-        <v>51</v>
+        <v>22</v>
       </c>
       <c r="I19" s="3" t="s">
         <v>23</v>
       </c>
       <c r="J19" s="3" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="K19" s="3" t="s">
-        <v>176</v>
+        <v>135</v>
       </c>
       <c r="L19" s="3" t="s">
-        <v>40</v>
+        <v>26</v>
       </c>
       <c r="M19" s="3" t="s">
-        <v>27</v>
+        <v>177</v>
       </c>
       <c r="N19" s="3" t="s">
         <v>28</v>
@@ -2300,51 +2282,51 @@
         <v>29</v>
       </c>
       <c r="P19" s="3" t="s">
-        <v>30</v>
+        <v>44</v>
       </c>
       <c r="Q19" s="3" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
     </row>
     <row r="20" spans="1:17" ht="12.75">
       <c r="A20" s="3" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="D20" s="3" t="s">
         <v>20</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>83</v>
+        <v>183</v>
       </c>
       <c r="G20" s="4">
-        <v>193000</v>
+        <v>189900</v>
       </c>
       <c r="H20" s="3" t="s">
         <v>22</v>
       </c>
       <c r="I20" s="3" t="s">
-        <v>23</v>
+        <v>143</v>
       </c>
       <c r="J20" s="3" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="K20" s="3" t="s">
-        <v>141</v>
+        <v>170</v>
       </c>
       <c r="L20" s="3" t="s">
-        <v>26</v>
+        <v>40</v>
       </c>
       <c r="M20" s="3" t="s">
-        <v>183</v>
+        <v>27</v>
       </c>
       <c r="N20" s="3" t="s">
         <v>28</v>
@@ -2353,45 +2335,45 @@
         <v>29</v>
       </c>
       <c r="P20" s="3" t="s">
-        <v>44</v>
+        <v>30</v>
       </c>
       <c r="Q20" s="3" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
     </row>
     <row r="21" spans="1:17" ht="12.75">
       <c r="A21" s="3" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="D21" s="3" t="s">
         <v>20</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="G21" s="4">
-        <v>189900</v>
+        <v>189000</v>
       </c>
       <c r="H21" s="3" t="s">
         <v>22</v>
       </c>
       <c r="I21" s="3" t="s">
-        <v>149</v>
+        <v>23</v>
       </c>
       <c r="J21" s="3" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="K21" s="3" t="s">
-        <v>176</v>
+        <v>192</v>
       </c>
       <c r="L21" s="3" t="s">
         <v>40</v>
@@ -2409,48 +2391,48 @@
         <v>30</v>
       </c>
       <c r="Q21" s="3" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
     </row>
     <row r="22" spans="1:17" ht="12.75">
       <c r="A22" s="3" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="D22" s="3" t="s">
         <v>20</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="F22" s="3" t="s">
         <v>196</v>
       </c>
       <c r="G22" s="4">
-        <v>189000</v>
+        <v>178000</v>
       </c>
       <c r="H22" s="3" t="s">
         <v>22</v>
       </c>
       <c r="I22" s="3" t="s">
-        <v>23</v>
+        <v>126</v>
       </c>
       <c r="J22" s="3" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="K22" s="3" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="L22" s="3" t="s">
         <v>40</v>
       </c>
       <c r="M22" s="3" t="s">
-        <v>27</v>
+        <v>200</v>
       </c>
       <c r="N22" s="3" t="s">
         <v>28</v>
@@ -2459,51 +2441,51 @@
         <v>29</v>
       </c>
       <c r="P22" s="3" t="s">
-        <v>30</v>
+        <v>119</v>
       </c>
       <c r="Q22" s="3" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="23" spans="1:17" ht="12.75">
       <c r="A23" s="3" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="D23" s="3" t="s">
         <v>20</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="G23" s="4">
-        <v>178000</v>
+        <v>177500</v>
       </c>
       <c r="H23" s="3" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="I23" s="3" t="s">
-        <v>132</v>
+        <v>37</v>
       </c>
       <c r="J23" s="3" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="K23" s="3" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="L23" s="3" t="s">
         <v>40</v>
       </c>
       <c r="M23" s="3" t="s">
-        <v>206</v>
+        <v>27</v>
       </c>
       <c r="N23" s="3" t="s">
         <v>28</v>
@@ -2512,157 +2494,157 @@
         <v>29</v>
       </c>
       <c r="P23" s="3" t="s">
-        <v>125</v>
+        <v>30</v>
       </c>
       <c r="Q23" s="3" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
     </row>
     <row r="24" spans="1:17" ht="12.75">
       <c r="A24" s="3" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="D24" s="3" t="s">
         <v>20</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="G24" s="4">
-        <v>177500</v>
+        <v>163000</v>
       </c>
       <c r="H24" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="I24" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I24" s="3" t="s">
-        <v>37</v>
-      </c>
       <c r="J24" s="3" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="K24" s="3" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="L24" s="3" t="s">
         <v>40</v>
       </c>
       <c r="M24" s="3" t="s">
-        <v>27</v>
+        <v>217</v>
       </c>
       <c r="N24" s="3" t="s">
-        <v>28</v>
+        <v>218</v>
       </c>
       <c r="O24" s="3" t="s">
-        <v>29</v>
+        <v>43</v>
       </c>
       <c r="P24" s="3" t="s">
-        <v>30</v>
+        <v>119</v>
       </c>
       <c r="Q24" s="3" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
     </row>
     <row r="25" spans="1:17" ht="12.75">
       <c r="A25" s="3" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="D25" s="3" t="s">
         <v>20</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="G25" s="4">
-        <v>163000</v>
+        <v>147000</v>
       </c>
       <c r="H25" s="3" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="I25" s="3" t="s">
-        <v>23</v>
+        <v>126</v>
       </c>
       <c r="J25" s="3" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="K25" s="3" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="L25" s="3" t="s">
-        <v>40</v>
+        <v>26</v>
       </c>
       <c r="M25" s="3" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="N25" s="3" t="s">
-        <v>224</v>
+        <v>28</v>
       </c>
       <c r="O25" s="3" t="s">
-        <v>43</v>
+        <v>29</v>
       </c>
       <c r="P25" s="3" t="s">
-        <v>125</v>
+        <v>44</v>
       </c>
       <c r="Q25" s="3" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
     </row>
     <row r="26" spans="1:17" ht="12.75">
       <c r="A26" s="3" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="D26" s="3" t="s">
         <v>20</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="G26" s="4">
-        <v>147000</v>
+        <v>146700</v>
       </c>
       <c r="H26" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="I26" s="3" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="J26" s="3" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="K26" s="3" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="L26" s="3" t="s">
         <v>26</v>
       </c>
       <c r="M26" s="3" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="N26" s="3" t="s">
         <v>28</v>
@@ -2671,92 +2653,92 @@
         <v>29</v>
       </c>
       <c r="P26" s="3" t="s">
-        <v>44</v>
+        <v>30</v>
       </c>
       <c r="Q26" s="3" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
     </row>
     <row r="27" spans="1:17" ht="12.75">
       <c r="A27" s="3" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="D27" s="3" t="s">
         <v>20</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="F27" s="3" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="G27" s="4">
-        <v>146700</v>
+        <v>108000</v>
       </c>
       <c r="H27" s="3" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="I27" s="3" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="J27" s="3" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="K27" s="3" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="L27" s="3" t="s">
-        <v>26</v>
+        <v>40</v>
       </c>
       <c r="M27" s="3" t="s">
-        <v>242</v>
+        <v>95</v>
       </c>
       <c r="N27" s="3" t="s">
         <v>28</v>
       </c>
       <c r="O27" s="3" t="s">
-        <v>29</v>
+        <v>43</v>
       </c>
       <c r="P27" s="3" t="s">
-        <v>30</v>
+        <v>44</v>
       </c>
       <c r="Q27" s="3" t="s">
-        <v>243</v>
+        <v>96</v>
       </c>
     </row>
     <row r="28" spans="1:17" ht="12.75">
       <c r="A28" s="3" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="D28" s="3" t="s">
         <v>20</v>
       </c>
       <c r="E28" s="3" t="s">
+        <v>248</v>
+      </c>
+      <c r="F28" s="3" t="s">
         <v>247</v>
       </c>
-      <c r="F28" s="3" t="s">
-        <v>248</v>
-      </c>
       <c r="G28" s="4">
-        <v>108000</v>
+        <v>107500</v>
       </c>
       <c r="H28" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="I28" s="3" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="J28" s="3" t="s">
         <v>249</v>
@@ -2768,60 +2750,60 @@
         <v>40</v>
       </c>
       <c r="M28" s="3" t="s">
-        <v>95</v>
+        <v>27</v>
       </c>
       <c r="N28" s="3" t="s">
         <v>28</v>
       </c>
       <c r="O28" s="3" t="s">
-        <v>43</v>
+        <v>29</v>
       </c>
       <c r="P28" s="3" t="s">
-        <v>44</v>
+        <v>30</v>
       </c>
       <c r="Q28" s="3" t="s">
-        <v>28</v>
+        <v>251</v>
       </c>
     </row>
     <row r="29" spans="1:17" ht="12.75">
       <c r="A29" s="3" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>253</v>
+        <v>231</v>
       </c>
       <c r="D29" s="3" t="s">
         <v>20</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>254</v>
+        <v>232</v>
       </c>
       <c r="F29" s="3" t="s">
-        <v>253</v>
+        <v>233</v>
       </c>
       <c r="G29" s="4">
-        <v>107500</v>
+        <v>87000</v>
       </c>
       <c r="H29" s="3" t="s">
         <v>22</v>
       </c>
       <c r="I29" s="3" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="J29" s="3" t="s">
+        <v>254</v>
+      </c>
+      <c r="K29" s="3" t="s">
         <v>255</v>
       </c>
-      <c r="K29" s="3" t="s">
+      <c r="L29" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="M29" s="3" t="s">
         <v>256</v>
-      </c>
-      <c r="L29" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="M29" s="3" t="s">
-        <v>27</v>
       </c>
       <c r="N29" s="3" t="s">
         <v>28</v>
@@ -2830,63 +2812,10 @@
         <v>29</v>
       </c>
       <c r="P29" s="3" t="s">
-        <v>30</v>
+        <v>44</v>
       </c>
       <c r="Q29" s="3" t="s">
         <v>257</v>
-      </c>
-    </row>
-    <row r="30" spans="1:17" ht="12.75">
-      <c r="A30" s="3" t="s">
-        <v>258</v>
-      </c>
-      <c r="B30" s="3" t="s">
-        <v>259</v>
-      </c>
-      <c r="C30" s="3" t="s">
-        <v>237</v>
-      </c>
-      <c r="D30" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="E30" s="3" t="s">
-        <v>238</v>
-      </c>
-      <c r="F30" s="3" t="s">
-        <v>239</v>
-      </c>
-      <c r="G30" s="4">
-        <v>87000</v>
-      </c>
-      <c r="H30" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="I30" s="3" t="s">
-        <v>132</v>
-      </c>
-      <c r="J30" s="3" t="s">
-        <v>260</v>
-      </c>
-      <c r="K30" s="3" t="s">
-        <v>261</v>
-      </c>
-      <c r="L30" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="M30" s="3" t="s">
-        <v>262</v>
-      </c>
-      <c r="N30" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="O30" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="P30" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="Q30" s="3" t="s">
-        <v>263</v>
       </c>
     </row>
   </sheetData>

</xml_diff>